<commit_message>
Update SVG assets for clarity and accuracy in visual representation
- Modified "The assistant with everything" SVG to reflect updated read/write pairing calculations.
- Added new "Bound Answer" SVG to illustrate independent trials and failure rates.
- Adjusted "Bound" SVG to clarify upper bound calculations and assumptions.
- Revised "Monkeys, then guards" SVG for improved visual flow and clarity on decision-making processes.
- Updated "Version Picker" SVG to correct version age and enhance user interface descriptions.
</commit_message>
<xml_diff>
--- a/artifacts/speaking-opportunity-research/results/consolidated/speaking-opportunity-rankings.xlsx
+++ b/artifacts/speaking-opportunity-research/results/consolidated/speaking-opportunity-rankings.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="1" r:id="R0f23d684844d4e6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="2" r:id="R94af9289fbf74fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All opportunities" sheetId="3" r:id="R29d8e5d16ea94025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Community routes" sheetId="4" r:id="Rc7dc7e9651a7416b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deadlines" sheetId="5" r:id="R3be088ebe4f846c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="1" r:id="Rf5f97dff473848c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="2" r:id="R5afbd66694e74839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All opportunities" sheetId="3" r:id="R39a32568344b4e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Community routes" sheetId="4" r:id="Rd868d726dbb04dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deadlines" sheetId="5" r:id="Rd8a84995167544de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -561,7 +561,7 @@
       <x:c r="F5" s="17"/>
       <x:c r="G5" s="17"/>
       <x:c r="H5" s="11" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="I5" s="11" t="n">
         <x:v>1</x:v>
@@ -700,7 +700,7 @@
         <x:v>46345.5</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="I8" s="12" t="n">
         <x:v>1</x:v>
@@ -745,7 +745,7 @@
       </x:c>
       <x:c r="G9" s="18"/>
       <x:c r="H9" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I9" s="12" t="n">
         <x:v>1</x:v>
@@ -790,7 +790,7 @@
       </x:c>
       <x:c r="G10" s="18"/>
       <x:c r="H10" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="I10" s="12" t="n">
         <x:v>1</x:v>
@@ -835,7 +835,7 @@
       </x:c>
       <x:c r="G11" s="18"/>
       <x:c r="H11" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I11" s="12" t="n">
         <x:v>1</x:v>
@@ -882,7 +882,7 @@
         <x:v>46283.5</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="I12" s="12" t="n">
         <x:v>2</x:v>
@@ -929,7 +929,7 @@
         <x:v>46283.5</x:v>
       </x:c>
       <x:c r="H13" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I13" s="12" t="n">
         <x:v>2</x:v>
@@ -974,7 +974,7 @@
       </x:c>
       <x:c r="G14" s="18"/>
       <x:c r="H14" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="I14" s="12" t="n">
         <x:v>1</x:v>
@@ -1019,7 +1019,7 @@
       </x:c>
       <x:c r="G15" s="18"/>
       <x:c r="H15" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I15" s="12" t="n">
         <x:v>1</x:v>
@@ -1064,7 +1064,7 @@
       </x:c>
       <x:c r="G16" s="18"/>
       <x:c r="H16" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I16" s="12" t="n">
         <x:v>1</x:v>
@@ -1107,7 +1107,7 @@
       <x:c r="F17" s="18"/>
       <x:c r="G17" s="18"/>
       <x:c r="H17" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I17" s="12" t="n">
         <x:v>1</x:v>
@@ -1152,7 +1152,7 @@
       </x:c>
       <x:c r="G18" s="18"/>
       <x:c r="H18" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I18" s="12" t="n">
         <x:v>1</x:v>
@@ -1199,7 +1199,7 @@
         <x:v>46367.5</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
-        <x:v>Rethinking Parallelization in the Agentic Era</x:v>
+        <x:v>Compute, Please (and a Receipt)</x:v>
       </x:c>
       <x:c r="I19" s="12" t="n">
         <x:v>1</x:v>
@@ -1244,7 +1244,7 @@
       </x:c>
       <x:c r="G20" s="18"/>
       <x:c r="H20" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I20" s="12" t="n">
         <x:v>1</x:v>
@@ -1289,7 +1289,7 @@
       </x:c>
       <x:c r="G21" s="18"/>
       <x:c r="H21" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I21" s="12" t="n">
         <x:v>1</x:v>
@@ -1381,7 +1381,7 @@
       </x:c>
       <x:c r="G23" s="18"/>
       <x:c r="H23" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I23" s="12" t="n">
         <x:v>1</x:v>
@@ -1469,7 +1469,7 @@
       </x:c>
       <x:c r="G25" s="18"/>
       <x:c r="H25" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I25" s="12" t="n">
         <x:v>1</x:v>
@@ -1514,7 +1514,7 @@
       </x:c>
       <x:c r="G26" s="18"/>
       <x:c r="H26" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I26" s="12" t="n">
         <x:v>1</x:v>
@@ -1608,7 +1608,7 @@
         <x:v>46271.5</x:v>
       </x:c>
       <x:c r="H28" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="I28" s="12" t="n">
         <x:v>1</x:v>
@@ -1655,7 +1655,7 @@
         <x:v>46300.5</x:v>
       </x:c>
       <x:c r="H29" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="I29" s="12" t="n">
         <x:v>1</x:v>
@@ -1700,7 +1700,7 @@
       </x:c>
       <x:c r="G30" s="18"/>
       <x:c r="H30" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I30" s="12" t="n">
         <x:v>1</x:v>
@@ -1743,7 +1743,7 @@
       <x:c r="F31" s="18"/>
       <x:c r="G31" s="18"/>
       <x:c r="H31" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I31" s="12" t="n">
         <x:v>1</x:v>
@@ -1788,7 +1788,7 @@
       </x:c>
       <x:c r="G32" s="18"/>
       <x:c r="H32" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I32" s="12" t="n">
         <x:v>1</x:v>
@@ -1835,7 +1835,7 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="H33" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="I33" s="12" t="n">
         <x:v>1</x:v>
@@ -1880,7 +1880,7 @@
       </x:c>
       <x:c r="G34" s="18"/>
       <x:c r="H34" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="I34" s="12" t="n">
         <x:v>1</x:v>
@@ -1925,7 +1925,7 @@
       </x:c>
       <x:c r="G35" s="18"/>
       <x:c r="H35" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I35" s="12" t="n">
         <x:v>1</x:v>
@@ -1970,7 +1970,7 @@
       </x:c>
       <x:c r="G36" s="18"/>
       <x:c r="H36" s="12" t="str">
-        <x:v>Rethinking Parallelization in the Agentic Era</x:v>
+        <x:v>Compute, Please (and a Receipt)</x:v>
       </x:c>
       <x:c r="I36" s="12" t="n">
         <x:v>1</x:v>
@@ -2109,7 +2109,7 @@
       </x:c>
       <x:c r="G39" s="18"/>
       <x:c r="H39" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="I39" s="12" t="n">
         <x:v>1</x:v>
@@ -2199,7 +2199,7 @@
       <x:c r="F41" s="18"/>
       <x:c r="G41" s="18"/>
       <x:c r="H41" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="I41" s="12" t="n">
         <x:v>1</x:v>
@@ -2242,7 +2242,7 @@
       <x:c r="F42" s="18"/>
       <x:c r="G42" s="18"/>
       <x:c r="H42" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="I42" s="12" t="n">
         <x:v>1</x:v>
@@ -2289,7 +2289,7 @@
         <x:v>46299.5</x:v>
       </x:c>
       <x:c r="H43" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="I43" s="12" t="n">
         <x:v>1</x:v>
@@ -2399,7 +2399,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23d40734336e4475"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7496edc0ddd4ef3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2710,7 +2710,7 @@
       </x:c>
       <x:c r="J5" s="17"/>
       <x:c r="K5" s="11" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L5" s="11" t="str"/>
       <x:c r="M5" s="11" t="n">
@@ -2934,7 +2934,7 @@
         <x:v>46345.5</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
         <x:v>benchmarks</x:v>
@@ -3010,7 +3010,7 @@
       </x:c>
       <x:c r="J9" s="18"/>
       <x:c r="K9" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str"/>
       <x:c r="M9" s="12" t="n">
@@ -3084,7 +3084,7 @@
       </x:c>
       <x:c r="J10" s="18"/>
       <x:c r="K10" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str"/>
       <x:c r="M10" s="12" t="n">
@@ -3156,7 +3156,7 @@
       </x:c>
       <x:c r="J11" s="18"/>
       <x:c r="K11" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L11" s="12" t="str"/>
       <x:c r="M11" s="12" t="n">
@@ -3232,10 +3232,10 @@
         <x:v>46283.5</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>parallelization</x:v>
+        <x:v>retrieval</x:v>
       </x:c>
       <x:c r="M12" s="12" t="n">
         <x:v>2</x:v>
@@ -3310,7 +3310,7 @@
         <x:v>46283.5</x:v>
       </x:c>
       <x:c r="K13" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
         <x:v>judgment</x:v>
@@ -3386,7 +3386,7 @@
       </x:c>
       <x:c r="J14" s="18"/>
       <x:c r="K14" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str"/>
       <x:c r="M14" s="12" t="n">
@@ -3460,7 +3460,7 @@
       </x:c>
       <x:c r="J15" s="18"/>
       <x:c r="K15" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str"/>
       <x:c r="M15" s="12" t="n">
@@ -3534,7 +3534,7 @@
       </x:c>
       <x:c r="J16" s="18"/>
       <x:c r="K16" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L16" s="12" t="str"/>
       <x:c r="M16" s="12" t="n">
@@ -3606,7 +3606,7 @@
       </x:c>
       <x:c r="J17" s="18"/>
       <x:c r="K17" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str"/>
       <x:c r="M17" s="12" t="n">
@@ -3680,7 +3680,7 @@
       </x:c>
       <x:c r="J18" s="18"/>
       <x:c r="K18" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str"/>
       <x:c r="M18" s="12" t="n">
@@ -3756,7 +3756,7 @@
         <x:v>46367.5</x:v>
       </x:c>
       <x:c r="K19" s="12" t="str">
-        <x:v>Rethinking Parallelization in the Agentic Era</x:v>
+        <x:v>Compute, Please (and a Receipt)</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -3832,7 +3832,7 @@
       </x:c>
       <x:c r="J20" s="18"/>
       <x:c r="K20" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str"/>
       <x:c r="M20" s="12" t="n">
@@ -3904,7 +3904,7 @@
       </x:c>
       <x:c r="J21" s="18"/>
       <x:c r="K21" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L21" s="12" t="str"/>
       <x:c r="M21" s="12" t="n">
@@ -4054,7 +4054,7 @@
       </x:c>
       <x:c r="J23" s="18"/>
       <x:c r="K23" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L23" s="12" t="str"/>
       <x:c r="M23" s="12" t="n">
@@ -4198,7 +4198,7 @@
       </x:c>
       <x:c r="J25" s="18"/>
       <x:c r="K25" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L25" s="12" t="str"/>
       <x:c r="M25" s="12" t="n">
@@ -4270,7 +4270,7 @@
       </x:c>
       <x:c r="J26" s="18"/>
       <x:c r="K26" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L26" s="12" t="str"/>
       <x:c r="M26" s="12" t="n">
@@ -4422,7 +4422,7 @@
         <x:v>46271.5</x:v>
       </x:c>
       <x:c r="K28" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L28" s="12" t="str"/>
       <x:c r="M28" s="12" t="n">
@@ -4498,7 +4498,7 @@
         <x:v>46300.5</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L29" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -4574,7 +4574,7 @@
       </x:c>
       <x:c r="J30" s="18"/>
       <x:c r="K30" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L30" s="12" t="str"/>
       <x:c r="M30" s="12" t="n">
@@ -4646,7 +4646,7 @@
       </x:c>
       <x:c r="J31" s="18"/>
       <x:c r="K31" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L31" s="12" t="str"/>
       <x:c r="M31" s="12" t="n">
@@ -4720,7 +4720,7 @@
       </x:c>
       <x:c r="J32" s="18"/>
       <x:c r="K32" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L32" s="12" t="str"/>
       <x:c r="M32" s="12" t="n">
@@ -4794,7 +4794,7 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="K33" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L33" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -4870,7 +4870,7 @@
       </x:c>
       <x:c r="J34" s="18"/>
       <x:c r="K34" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L34" s="12" t="str"/>
       <x:c r="M34" s="12" t="n">
@@ -4942,7 +4942,7 @@
       </x:c>
       <x:c r="J35" s="18"/>
       <x:c r="K35" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L35" s="12" t="str"/>
       <x:c r="M35" s="12" t="n">
@@ -5016,7 +5016,7 @@
       </x:c>
       <x:c r="J36" s="18"/>
       <x:c r="K36" s="12" t="str">
-        <x:v>Rethinking Parallelization in the Agentic Era</x:v>
+        <x:v>Compute, Please (and a Receipt)</x:v>
       </x:c>
       <x:c r="L36" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -5246,7 +5246,7 @@
       </x:c>
       <x:c r="J39" s="18"/>
       <x:c r="K39" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L39" s="12" t="str"/>
       <x:c r="M39" s="12" t="n">
@@ -5396,7 +5396,7 @@
       </x:c>
       <x:c r="J41" s="18"/>
       <x:c r="K41" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L41" s="12" t="str"/>
       <x:c r="M41" s="12" t="n">
@@ -5466,7 +5466,7 @@
       </x:c>
       <x:c r="J42" s="18"/>
       <x:c r="K42" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L42" s="12" t="str"/>
       <x:c r="M42" s="12" t="n">
@@ -5540,7 +5540,7 @@
         <x:v>46299.5</x:v>
       </x:c>
       <x:c r="K43" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L43" s="12" t="str"/>
       <x:c r="M43" s="12" t="n">
@@ -5692,7 +5692,7 @@
         <x:v>46366.5</x:v>
       </x:c>
       <x:c r="K45" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L45" s="12" t="str">
         <x:v>judgment</x:v>
@@ -5844,7 +5844,7 @@
       </x:c>
       <x:c r="J47" s="18"/>
       <x:c r="K47" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L47" s="12" t="str"/>
       <x:c r="M47" s="12" t="n">
@@ -5914,7 +5914,7 @@
       </x:c>
       <x:c r="J48" s="18"/>
       <x:c r="K48" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L48" s="12" t="str"/>
       <x:c r="M48" s="12" t="n">
@@ -5988,7 +5988,7 @@
       </x:c>
       <x:c r="J49" s="18"/>
       <x:c r="K49" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L49" s="12" t="str"/>
       <x:c r="M49" s="12" t="n">
@@ -6064,7 +6064,7 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="K50" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L50" s="12" t="str">
         <x:v>adaptive-systems</x:v>
@@ -6138,7 +6138,7 @@
       </x:c>
       <x:c r="J51" s="18"/>
       <x:c r="K51" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L51" s="12" t="str"/>
       <x:c r="M51" s="12" t="n">
@@ -6208,7 +6208,7 @@
       </x:c>
       <x:c r="J52" s="18"/>
       <x:c r="K52" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L52" s="12" t="str"/>
       <x:c r="M52" s="12" t="n">
@@ -6280,7 +6280,7 @@
       </x:c>
       <x:c r="J53" s="18"/>
       <x:c r="K53" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L53" s="12" t="str"/>
       <x:c r="M53" s="12" t="n">
@@ -6356,7 +6356,7 @@
         <x:v>46299.5</x:v>
       </x:c>
       <x:c r="K54" s="12" t="str">
-        <x:v>Rethinking Parallelization in the Agentic Era</x:v>
+        <x:v>Compute, Please (and a Receipt)</x:v>
       </x:c>
       <x:c r="L54" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -6434,7 +6434,7 @@
         <x:v>46327.5</x:v>
       </x:c>
       <x:c r="K55" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L55" s="12" t="str">
         <x:v>retrieval</x:v>
@@ -6582,7 +6582,7 @@
       </x:c>
       <x:c r="J57" s="18"/>
       <x:c r="K57" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L57" s="12" t="str"/>
       <x:c r="M57" s="12" t="n">
@@ -6654,7 +6654,7 @@
       </x:c>
       <x:c r="J58" s="18"/>
       <x:c r="K58" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L58" s="12" t="str"/>
       <x:c r="M58" s="12" t="n">
@@ -6728,7 +6728,7 @@
       </x:c>
       <x:c r="J59" s="18"/>
       <x:c r="K59" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L59" s="12" t="str"/>
       <x:c r="M59" s="12" t="n">
@@ -6802,7 +6802,7 @@
       </x:c>
       <x:c r="J60" s="18"/>
       <x:c r="K60" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L60" s="12" t="str"/>
       <x:c r="M60" s="12" t="n">
@@ -6878,7 +6878,7 @@
         <x:v>46367.5</x:v>
       </x:c>
       <x:c r="K61" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L61" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -7032,7 +7032,7 @@
       </x:c>
       <x:c r="J63" s="18"/>
       <x:c r="K63" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L63" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -7108,7 +7108,7 @@
       </x:c>
       <x:c r="J64" s="18"/>
       <x:c r="K64" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L64" s="12" t="str">
         <x:v>judgment</x:v>
@@ -7184,7 +7184,7 @@
       </x:c>
       <x:c r="J65" s="18"/>
       <x:c r="K65" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L65" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -7260,7 +7260,7 @@
       </x:c>
       <x:c r="J66" s="18"/>
       <x:c r="K66" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L66" s="12" t="str"/>
       <x:c r="M66" s="12" t="n">
@@ -7410,7 +7410,7 @@
       </x:c>
       <x:c r="J68" s="18"/>
       <x:c r="K68" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L68" s="12" t="str"/>
       <x:c r="M68" s="12" t="n">
@@ -7482,7 +7482,7 @@
       </x:c>
       <x:c r="J69" s="18"/>
       <x:c r="K69" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L69" s="12" t="str"/>
       <x:c r="M69" s="12" t="n">
@@ -7556,7 +7556,7 @@
       </x:c>
       <x:c r="J70" s="18"/>
       <x:c r="K70" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L70" s="12" t="str"/>
       <x:c r="M70" s="12" t="n">
@@ -7626,7 +7626,7 @@
       </x:c>
       <x:c r="J71" s="18"/>
       <x:c r="K71" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L71" s="12" t="str"/>
       <x:c r="M71" s="12" t="n">
@@ -7776,7 +7776,7 @@
       </x:c>
       <x:c r="J73" s="18"/>
       <x:c r="K73" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L73" s="12" t="str"/>
       <x:c r="M73" s="12" t="n">
@@ -7848,7 +7848,7 @@
       </x:c>
       <x:c r="J74" s="18"/>
       <x:c r="K74" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L74" s="12" t="str"/>
       <x:c r="M74" s="12" t="n">
@@ -7918,7 +7918,7 @@
       </x:c>
       <x:c r="J75" s="18"/>
       <x:c r="K75" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L75" s="12" t="str"/>
       <x:c r="M75" s="12" t="n">
@@ -7992,7 +7992,7 @@
         <x:v>46388.5</x:v>
       </x:c>
       <x:c r="K76" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L76" s="12" t="str">
         <x:v>retrieval</x:v>
@@ -8070,7 +8070,7 @@
         <x:v>46295.5</x:v>
       </x:c>
       <x:c r="K77" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L77" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -8146,7 +8146,7 @@
       </x:c>
       <x:c r="J78" s="18"/>
       <x:c r="K78" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L78" s="12" t="str"/>
       <x:c r="M78" s="12" t="n">
@@ -8218,7 +8218,7 @@
       </x:c>
       <x:c r="J79" s="18"/>
       <x:c r="K79" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L79" s="12" t="str"/>
       <x:c r="M79" s="12" t="n">
@@ -8292,7 +8292,7 @@
       </x:c>
       <x:c r="J80" s="18"/>
       <x:c r="K80" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L80" s="12" t="str"/>
       <x:c r="M80" s="12" t="n">
@@ -8364,7 +8364,7 @@
       </x:c>
       <x:c r="J81" s="18"/>
       <x:c r="K81" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L81" s="12" t="str"/>
       <x:c r="M81" s="12" t="n">
@@ -8440,7 +8440,7 @@
         <x:v>46310.5</x:v>
       </x:c>
       <x:c r="K82" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L82" s="12" t="str">
         <x:v>judgment</x:v>
@@ -8518,7 +8518,7 @@
         <x:v>46374.5</x:v>
       </x:c>
       <x:c r="K83" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L83" s="12" t="str"/>
       <x:c r="M83" s="12" t="n">
@@ -8670,7 +8670,7 @@
         <x:v>46279.5</x:v>
       </x:c>
       <x:c r="K85" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L85" s="12" t="str"/>
       <x:c r="M85" s="12" t="n">
@@ -8740,7 +8740,7 @@
       </x:c>
       <x:c r="J86" s="18"/>
       <x:c r="K86" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L86" s="12" t="str"/>
       <x:c r="M86" s="12" t="n">
@@ -8814,7 +8814,7 @@
         <x:v>46307.5</x:v>
       </x:c>
       <x:c r="K87" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L87" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -8958,7 +8958,7 @@
       </x:c>
       <x:c r="J89" s="18"/>
       <x:c r="K89" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L89" s="12" t="str"/>
       <x:c r="M89" s="12" t="n">
@@ -9028,7 +9028,7 @@
       </x:c>
       <x:c r="J90" s="18"/>
       <x:c r="K90" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L90" s="12" t="str"/>
       <x:c r="M90" s="12" t="n">
@@ -9100,7 +9100,7 @@
       </x:c>
       <x:c r="J91" s="18"/>
       <x:c r="K91" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L91" s="12" t="str"/>
       <x:c r="M91" s="12" t="n">
@@ -9252,7 +9252,7 @@
         <x:v>46313.5</x:v>
       </x:c>
       <x:c r="K93" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L93" s="12" t="str"/>
       <x:c r="M93" s="12" t="n">
@@ -9328,7 +9328,7 @@
         <x:v>46318.5</x:v>
       </x:c>
       <x:c r="K94" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L94" s="12" t="str">
         <x:v>retrieval</x:v>
@@ -9404,7 +9404,7 @@
       </x:c>
       <x:c r="J95" s="18"/>
       <x:c r="K95" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L95" s="12" t="str"/>
       <x:c r="M95" s="12" t="n">
@@ -9478,7 +9478,7 @@
       </x:c>
       <x:c r="J96" s="18"/>
       <x:c r="K96" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L96" s="12" t="str"/>
       <x:c r="M96" s="12" t="n">
@@ -9548,7 +9548,7 @@
       </x:c>
       <x:c r="J97" s="18"/>
       <x:c r="K97" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L97" s="12" t="str"/>
       <x:c r="M97" s="12" t="n">
@@ -9624,7 +9624,7 @@
         <x:v>46310.5</x:v>
       </x:c>
       <x:c r="K98" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L98" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -9700,7 +9700,7 @@
       </x:c>
       <x:c r="J99" s="18"/>
       <x:c r="K99" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L99" s="12" t="str"/>
       <x:c r="M99" s="12" t="n">
@@ -9848,7 +9848,7 @@
       </x:c>
       <x:c r="J101" s="18"/>
       <x:c r="K101" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L101" s="12" t="str"/>
       <x:c r="M101" s="12" t="n">
@@ -9992,7 +9992,7 @@
       </x:c>
       <x:c r="J103" s="18"/>
       <x:c r="K103" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L103" s="12" t="str"/>
       <x:c r="M103" s="12" t="n">
@@ -10064,7 +10064,7 @@
       </x:c>
       <x:c r="J104" s="18"/>
       <x:c r="K104" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L104" s="12" t="str"/>
       <x:c r="M104" s="12" t="n">
@@ -10140,7 +10140,7 @@
         <x:v>46306.5</x:v>
       </x:c>
       <x:c r="K105" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L105" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -10218,7 +10218,7 @@
         <x:v>46313.5</x:v>
       </x:c>
       <x:c r="K106" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L106" s="12" t="str">
         <x:v>adaptive-systems</x:v>
@@ -10370,7 +10370,7 @@
       </x:c>
       <x:c r="J108" s="18"/>
       <x:c r="K108" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L108" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -10444,7 +10444,7 @@
       </x:c>
       <x:c r="J109" s="18"/>
       <x:c r="K109" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L109" s="12" t="str"/>
       <x:c r="M109" s="12" t="n">
@@ -10518,7 +10518,7 @@
       </x:c>
       <x:c r="J110" s="18"/>
       <x:c r="K110" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L110" s="12" t="str">
         <x:v>judgment</x:v>
@@ -10592,7 +10592,7 @@
       </x:c>
       <x:c r="J111" s="18"/>
       <x:c r="K111" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L111" s="12" t="str"/>
       <x:c r="M111" s="12" t="n">
@@ -10668,7 +10668,7 @@
         <x:v>46297.5</x:v>
       </x:c>
       <x:c r="K112" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L112" s="12" t="str"/>
       <x:c r="M112" s="12" t="n">
@@ -10744,7 +10744,7 @@
         <x:v>46369.5</x:v>
       </x:c>
       <x:c r="K113" s="12" t="str">
-        <x:v>Rethinking Parallelization in the Agentic Era</x:v>
+        <x:v>Compute, Please (and a Receipt)</x:v>
       </x:c>
       <x:c r="L113" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -10970,7 +10970,7 @@
         <x:v>46313.5</x:v>
       </x:c>
       <x:c r="K116" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L116" s="12" t="str">
         <x:v>adaptive-systems</x:v>
@@ -11048,7 +11048,7 @@
         <x:v>46306.5</x:v>
       </x:c>
       <x:c r="K117" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L117" s="12" t="str">
         <x:v>retrieval</x:v>
@@ -11198,7 +11198,7 @@
       </x:c>
       <x:c r="J119" s="18"/>
       <x:c r="K119" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="L119" s="12" t="str"/>
       <x:c r="M119" s="12" t="n">
@@ -11346,7 +11346,7 @@
       </x:c>
       <x:c r="J121" s="18"/>
       <x:c r="K121" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L121" s="12" t="str"/>
       <x:c r="M121" s="12" t="n">
@@ -11420,7 +11420,7 @@
       </x:c>
       <x:c r="J122" s="18"/>
       <x:c r="K122" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L122" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -11494,7 +11494,7 @@
       </x:c>
       <x:c r="J123" s="18"/>
       <x:c r="K123" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L123" s="12" t="str"/>
       <x:c r="M123" s="12" t="n">
@@ -11566,7 +11566,7 @@
       </x:c>
       <x:c r="J124" s="18"/>
       <x:c r="K124" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L124" s="12" t="str"/>
       <x:c r="M124" s="12" t="n">
@@ -11638,7 +11638,7 @@
       </x:c>
       <x:c r="J125" s="18"/>
       <x:c r="K125" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L125" s="12" t="str">
         <x:v>judgment</x:v>
@@ -11712,7 +11712,7 @@
       </x:c>
       <x:c r="J126" s="18"/>
       <x:c r="K126" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L126" s="12" t="str"/>
       <x:c r="M126" s="12" t="n">
@@ -11784,7 +11784,7 @@
       </x:c>
       <x:c r="J127" s="18"/>
       <x:c r="K127" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L127" s="12" t="str"/>
       <x:c r="M127" s="12" t="n">
@@ -11858,7 +11858,7 @@
       </x:c>
       <x:c r="J128" s="18"/>
       <x:c r="K128" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L128" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -11936,7 +11936,7 @@
         <x:v>46313.5</x:v>
       </x:c>
       <x:c r="K129" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L129" s="12" t="str">
         <x:v>adaptive-systems</x:v>
@@ -12014,7 +12014,7 @@
         <x:v>46326.5</x:v>
       </x:c>
       <x:c r="K130" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L130" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -12090,7 +12090,7 @@
       </x:c>
       <x:c r="J131" s="18"/>
       <x:c r="K131" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="L131" s="12" t="str"/>
       <x:c r="M131" s="12" t="n">
@@ -12160,7 +12160,7 @@
       </x:c>
       <x:c r="J132" s="18"/>
       <x:c r="K132" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L132" s="12" t="str"/>
       <x:c r="M132" s="12" t="n">
@@ -12232,7 +12232,7 @@
       </x:c>
       <x:c r="J133" s="18"/>
       <x:c r="K133" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L133" s="12" t="str"/>
       <x:c r="M133" s="12" t="n">
@@ -12458,7 +12458,7 @@
         <x:v>46296.5</x:v>
       </x:c>
       <x:c r="K136" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L136" s="12" t="str"/>
       <x:c r="M136" s="12" t="n">
@@ -12604,7 +12604,7 @@
       </x:c>
       <x:c r="J138" s="18"/>
       <x:c r="K138" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L138" s="12" t="str">
         <x:v>failure-improvement</x:v>
@@ -12680,7 +12680,7 @@
       </x:c>
       <x:c r="J139" s="18"/>
       <x:c r="K139" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L139" s="12" t="str"/>
       <x:c r="M139" s="12" t="n">
@@ -12752,7 +12752,7 @@
       </x:c>
       <x:c r="J140" s="18"/>
       <x:c r="K140" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L140" s="12" t="str"/>
       <x:c r="M140" s="12" t="n">
@@ -12824,7 +12824,7 @@
       </x:c>
       <x:c r="J141" s="18"/>
       <x:c r="K141" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L141" s="12" t="str"/>
       <x:c r="M141" s="12" t="n">
@@ -12896,7 +12896,7 @@
       </x:c>
       <x:c r="J142" s="18"/>
       <x:c r="K142" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L142" s="12" t="str"/>
       <x:c r="M142" s="12" t="n">
@@ -12968,7 +12968,7 @@
       </x:c>
       <x:c r="J143" s="18"/>
       <x:c r="K143" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L143" s="12" t="str"/>
       <x:c r="M143" s="12" t="n">
@@ -13118,7 +13118,7 @@
       </x:c>
       <x:c r="J145" s="18"/>
       <x:c r="K145" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L145" s="12" t="str"/>
       <x:c r="M145" s="12" t="n">
@@ -13194,7 +13194,7 @@
         <x:v>46325.5</x:v>
       </x:c>
       <x:c r="K146" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L146" s="12" t="str"/>
       <x:c r="M146" s="12" t="n">
@@ -13270,7 +13270,7 @@
         <x:v>46325.5</x:v>
       </x:c>
       <x:c r="K147" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L147" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -13344,7 +13344,7 @@
       </x:c>
       <x:c r="J148" s="18"/>
       <x:c r="K148" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L148" s="12" t="str"/>
       <x:c r="M148" s="12" t="n">
@@ -13420,7 +13420,7 @@
         <x:v>46304.5</x:v>
       </x:c>
       <x:c r="K149" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L149" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -13498,7 +13498,7 @@
         <x:v>46290.5</x:v>
       </x:c>
       <x:c r="K150" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L150" s="12" t="str"/>
       <x:c r="M150" s="12" t="n">
@@ -13572,7 +13572,7 @@
       </x:c>
       <x:c r="J151" s="18"/>
       <x:c r="K151" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L151" s="12" t="str"/>
       <x:c r="M151" s="12" t="n">
@@ -13648,7 +13648,7 @@
         <x:v>46295.5</x:v>
       </x:c>
       <x:c r="K152" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L152" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -13724,7 +13724,7 @@
       </x:c>
       <x:c r="J153" s="18"/>
       <x:c r="K153" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L153" s="12" t="str"/>
       <x:c r="M153" s="12" t="n">
@@ -13798,7 +13798,7 @@
         <x:v>46296.5</x:v>
       </x:c>
       <x:c r="K154" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L154" s="12" t="str"/>
       <x:c r="M154" s="12" t="n">
@@ -13872,7 +13872,7 @@
       </x:c>
       <x:c r="J155" s="18"/>
       <x:c r="K155" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L155" s="12" t="str"/>
       <x:c r="M155" s="12" t="n">
@@ -13944,7 +13944,7 @@
       </x:c>
       <x:c r="J156" s="18"/>
       <x:c r="K156" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L156" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -14020,7 +14020,7 @@
       </x:c>
       <x:c r="J157" s="18"/>
       <x:c r="K157" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L157" s="12" t="str"/>
       <x:c r="M157" s="12" t="n">
@@ -14092,7 +14092,7 @@
       </x:c>
       <x:c r="J158" s="18"/>
       <x:c r="K158" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L158" s="12" t="str"/>
       <x:c r="M158" s="12" t="n">
@@ -14168,7 +14168,7 @@
         <x:v>46346.5</x:v>
       </x:c>
       <x:c r="K159" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L159" s="12" t="str"/>
       <x:c r="M159" s="12" t="n">
@@ -14244,7 +14244,7 @@
         <x:v>46376.5</x:v>
       </x:c>
       <x:c r="K160" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L160" s="12" t="str"/>
       <x:c r="M160" s="12" t="n">
@@ -14318,7 +14318,7 @@
       </x:c>
       <x:c r="J161" s="18"/>
       <x:c r="K161" s="12" t="str">
-        <x:v>Code Is Cheap. Judgment Is Expensive.</x:v>
+        <x:v>Turn Your Thinkin' Tokens Up to 11</x:v>
       </x:c>
       <x:c r="L161" s="12" t="str">
         <x:v>product-engineering</x:v>
@@ -14394,7 +14394,7 @@
       </x:c>
       <x:c r="J162" s="18"/>
       <x:c r="K162" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="L162" s="12" t="str">
         <x:v>parallelization</x:v>
@@ -14470,7 +14470,7 @@
       </x:c>
       <x:c r="J163" s="18"/>
       <x:c r="K163" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L163" s="12" t="str"/>
       <x:c r="M163" s="12" t="n">
@@ -14622,7 +14622,7 @@
       </x:c>
       <x:c r="J165" s="18"/>
       <x:c r="K165" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="L165" s="12" t="str"/>
       <x:c r="M165" s="12" t="n">
@@ -14770,7 +14770,7 @@
       </x:c>
       <x:c r="J167" s="18"/>
       <x:c r="K167" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="L167" s="12" t="str"/>
       <x:c r="M167" s="12" t="n">
@@ -14920,7 +14920,7 @@
       </x:c>
       <x:c r="J169" s="18"/>
       <x:c r="K169" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="L169" s="12" t="str"/>
       <x:c r="M169" s="12" t="n">
@@ -15056,7 +15056,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84548452d1644a9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2c4736550844c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15158,7 +15158,7 @@
       </x:c>
       <x:c r="E5" s="17"/>
       <x:c r="F5" s="11" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G5" s="11" t="n">
         <x:v>1</x:v>
@@ -15238,7 +15238,7 @@
         <x:v>46282.5</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G7" s="12" t="n">
         <x:v>1</x:v>
@@ -15279,7 +15279,7 @@
         <x:v>46310.5</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G8" s="12" t="n">
         <x:v>1</x:v>
@@ -15318,7 +15318,7 @@
         <x:v>46273.5</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G9" s="12" t="n">
         <x:v>1</x:v>
@@ -15359,7 +15359,7 @@
         <x:v>46294.5</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G10" s="12" t="n">
         <x:v>2</x:v>
@@ -15400,7 +15400,7 @@
         <x:v>46282.5</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G11" s="12" t="n">
         <x:v>2</x:v>
@@ -15439,7 +15439,7 @@
       </x:c>
       <x:c r="E12" s="18"/>
       <x:c r="F12" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G12" s="12" t="n">
         <x:v>2</x:v>
@@ -15480,7 +15480,7 @@
         <x:v>46289.5</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G13" s="12" t="n">
         <x:v>1</x:v>
@@ -15521,7 +15521,7 @@
         <x:v>46279.5</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G14" s="12" t="n">
         <x:v>2</x:v>
@@ -15560,7 +15560,7 @@
         <x:v>46281.5</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G15" s="12" t="n">
         <x:v>2</x:v>
@@ -15599,7 +15599,7 @@
         <x:v>46278.5</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G16" s="12" t="n">
         <x:v>1</x:v>
@@ -15677,7 +15677,7 @@
         <x:v>46287.5</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G18" s="12" t="n">
         <x:v>2</x:v>
@@ -15716,7 +15716,7 @@
         <x:v>46288.5</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G19" s="12" t="n">
         <x:v>2</x:v>
@@ -15755,7 +15755,7 @@
         <x:v>46280.5</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G20" s="12" t="n">
         <x:v>3</x:v>
@@ -15794,7 +15794,7 @@
       </x:c>
       <x:c r="E21" s="18"/>
       <x:c r="F21" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G21" s="12" t="n">
         <x:v>3</x:v>
@@ -15835,7 +15835,7 @@
         <x:v>46280.5</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G22" s="12" t="n">
         <x:v>1</x:v>
@@ -15874,7 +15874,7 @@
         <x:v>46284.5</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G23" s="12" t="n">
         <x:v>1</x:v>
@@ -15913,7 +15913,7 @@
       </x:c>
       <x:c r="E24" s="18"/>
       <x:c r="F24" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="G24" s="12" t="n">
         <x:v>2</x:v>
@@ -15950,7 +15950,7 @@
       </x:c>
       <x:c r="E25" s="18"/>
       <x:c r="F25" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G25" s="12" t="n">
         <x:v>2</x:v>
@@ -15989,7 +15989,7 @@
         <x:v>46287.5</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G26" s="12" t="n">
         <x:v>3</x:v>
@@ -16026,7 +16026,7 @@
       </x:c>
       <x:c r="E27" s="18"/>
       <x:c r="F27" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G27" s="12" t="n">
         <x:v>3</x:v>
@@ -16067,7 +16067,7 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G28" s="12" t="n">
         <x:v>3</x:v>
@@ -16106,7 +16106,7 @@
       </x:c>
       <x:c r="E29" s="18"/>
       <x:c r="F29" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G29" s="12" t="n">
         <x:v>1</x:v>
@@ -16143,7 +16143,7 @@
       </x:c>
       <x:c r="E30" s="18"/>
       <x:c r="F30" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G30" s="12" t="n">
         <x:v>4</x:v>
@@ -16182,7 +16182,7 @@
       </x:c>
       <x:c r="E31" s="18"/>
       <x:c r="F31" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="G31" s="12" t="n">
         <x:v>4</x:v>
@@ -16262,7 +16262,7 @@
       </x:c>
       <x:c r="E33" s="18"/>
       <x:c r="F33" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="G33" s="12" t="n">
         <x:v>2</x:v>
@@ -16301,7 +16301,7 @@
         <x:v>46284.5</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G34" s="12" t="n">
         <x:v>2</x:v>
@@ -16342,7 +16342,7 @@
         <x:v>46284.5</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G35" s="12" t="n">
         <x:v>3</x:v>
@@ -16381,7 +16381,7 @@
       </x:c>
       <x:c r="E36" s="18"/>
       <x:c r="F36" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G36" s="12" t="n">
         <x:v>3</x:v>
@@ -16422,7 +16422,7 @@
         <x:v>46279.5</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G37" s="12" t="n">
         <x:v>3</x:v>
@@ -16459,7 +16459,7 @@
       </x:c>
       <x:c r="E38" s="18"/>
       <x:c r="F38" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G38" s="12" t="n">
         <x:v>3</x:v>
@@ -16498,7 +16498,7 @@
       </x:c>
       <x:c r="E39" s="18"/>
       <x:c r="F39" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G39" s="12" t="n">
         <x:v>2</x:v>
@@ -16537,7 +16537,7 @@
         <x:v>46277.5</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G40" s="12" t="n">
         <x:v>4</x:v>
@@ -16578,7 +16578,7 @@
         <x:v>46277.5</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G41" s="12" t="n">
         <x:v>4</x:v>
@@ -16617,7 +16617,7 @@
       </x:c>
       <x:c r="E42" s="18"/>
       <x:c r="F42" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G42" s="12" t="n">
         <x:v>1</x:v>
@@ -16656,7 +16656,7 @@
       </x:c>
       <x:c r="E43" s="18"/>
       <x:c r="F43" s="12" t="str">
-        <x:v>Cry Me a Free Tier</x:v>
+        <x:v>Buy Me a Free Tier</x:v>
       </x:c>
       <x:c r="G43" s="12" t="n">
         <x:v>3</x:v>
@@ -16730,7 +16730,7 @@
       </x:c>
       <x:c r="E45" s="18"/>
       <x:c r="F45" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="G45" s="12" t="n">
         <x:v>4</x:v>
@@ -16767,7 +16767,7 @@
       </x:c>
       <x:c r="E46" s="18"/>
       <x:c r="F46" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G46" s="12" t="n">
         <x:v>4</x:v>
@@ -16808,7 +16808,7 @@
         <x:v>46277.5</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G47" s="12" t="n">
         <x:v>5</x:v>
@@ -16849,7 +16849,7 @@
         <x:v>46529.5</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="G48" s="12" t="n">
         <x:v>5</x:v>
@@ -16886,7 +16886,7 @@
       </x:c>
       <x:c r="E49" s="18"/>
       <x:c r="F49" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G49" s="12" t="n">
         <x:v>2</x:v>
@@ -16925,7 +16925,7 @@
       </x:c>
       <x:c r="E50" s="18"/>
       <x:c r="F50" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G50" s="12" t="n">
         <x:v>3</x:v>
@@ -16962,7 +16962,7 @@
       </x:c>
       <x:c r="E51" s="18"/>
       <x:c r="F51" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G51" s="12" t="n">
         <x:v>3</x:v>
@@ -17001,7 +17001,7 @@
       </x:c>
       <x:c r="E52" s="18"/>
       <x:c r="F52" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G52" s="12" t="n">
         <x:v>3</x:v>
@@ -17040,7 +17040,7 @@
       </x:c>
       <x:c r="E53" s="18"/>
       <x:c r="F53" s="12" t="str">
-        <x:v>From RAGs to Retrievals</x:v>
+        <x:v>Three Search Methods in a Fundable Trenchcoat</x:v>
       </x:c>
       <x:c r="G53" s="12" t="n">
         <x:v>1</x:v>
@@ -17081,7 +17081,7 @@
         <x:v>46441.5</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>Stop Looking at My Benchmarks</x:v>
+        <x:v>Stop Looking at My Benchmarks… Get Your Own!</x:v>
       </x:c>
       <x:c r="G54" s="12" t="n">
         <x:v>5</x:v>
@@ -17118,7 +17118,7 @@
       </x:c>
       <x:c r="E55" s="18"/>
       <x:c r="F55" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G55" s="12" t="n">
         <x:v>2</x:v>
@@ -17157,7 +17157,7 @@
       </x:c>
       <x:c r="E56" s="18"/>
       <x:c r="F56" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G56" s="12" t="n">
         <x:v>3</x:v>
@@ -17196,7 +17196,7 @@
       </x:c>
       <x:c r="E57" s="18"/>
       <x:c r="F57" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G57" s="12" t="n">
         <x:v>3</x:v>
@@ -17237,7 +17237,7 @@
         <x:v>46601.5</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
-        <x:v>The Future of Product Engineering</x:v>
+        <x:v>Break the Mirror on Purpose</x:v>
       </x:c>
       <x:c r="G58" s="12" t="n">
         <x:v>5</x:v>
@@ -17274,7 +17274,7 @@
       </x:c>
       <x:c r="E59" s="18"/>
       <x:c r="F59" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G59" s="12" t="n">
         <x:v>2</x:v>
@@ -17313,7 +17313,7 @@
       </x:c>
       <x:c r="E60" s="18"/>
       <x:c r="F60" s="12" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G60" s="12" t="n">
         <x:v>2</x:v>
@@ -17352,7 +17352,7 @@
       </x:c>
       <x:c r="E61" s="18"/>
       <x:c r="F61" s="12" t="str">
-        <x:v>Building Adaptive &amp; Dynamic AI Systems</x:v>
+        <x:v>Conjure Exactly Enough</x:v>
       </x:c>
       <x:c r="G61" s="12" t="n">
         <x:v>3</x:v>
@@ -17391,7 +17391,7 @@
       </x:c>
       <x:c r="E62" s="19"/>
       <x:c r="F62" s="13" t="str">
-        <x:v>Automating Improvement From Failure</x:v>
+        <x:v>The Pager Cried Wolf</x:v>
       </x:c>
       <x:c r="G62" s="13" t="n">
         <x:v>4</x:v>
@@ -17418,7 +17418,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffa34e4360b842b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7985482b704449a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22887,7 +22887,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R623dd0837dbb4544"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f7243a31c4e4547"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>